<commit_message>
- change paths - softcoding saving section create new dataframes and xlsxs (due to extended 13 years lai reference period)
</commit_message>
<xml_diff>
--- a/output/differences_absolute_regional.xlsx
+++ b/output/differences_absolute_regional.xlsx
@@ -428,10 +428,10 @@
         <v>0.01320400737437266</v>
       </c>
       <c r="G2">
-        <v>0.5110358817090557</v>
+        <v>0.5395974520831248</v>
       </c>
       <c r="H2">
-        <v>-0.05679894179894207</v>
+        <v>-0.05559939134939196</v>
       </c>
       <c r="I2" s="2">
         <v>41395</v>
@@ -457,10 +457,10 @@
         <v>-0.01106962491966235</v>
       </c>
       <c r="G3">
-        <v>0.174290646004291</v>
+        <v>0.1529515865576285</v>
       </c>
       <c r="H3">
-        <v>0.00948331736909136</v>
+        <v>0.04592384983045905</v>
       </c>
       <c r="I3" s="2">
         <v>41426</v>
@@ -486,10 +486,10 @@
         <v>-0.01300880110686986</v>
       </c>
       <c r="G4">
-        <v>0.3130461507358895</v>
+        <v>0.3843258234519102</v>
       </c>
       <c r="H4">
-        <v>0.337681216931216</v>
+        <v>0.3441054131054129</v>
       </c>
       <c r="I4" s="2">
         <v>41456</v>
@@ -515,10 +515,10 @@
         <v>0.00674705508873219</v>
       </c>
       <c r="G5">
-        <v>-0.02555955109573094</v>
+        <v>-0.05216796723675587</v>
       </c>
       <c r="H5">
-        <v>-0.03907462522045835</v>
+        <v>-0.06788997884831316</v>
       </c>
       <c r="I5" s="2">
         <v>41487</v>
@@ -544,10 +544,10 @@
         <v>0.01075174437662829</v>
       </c>
       <c r="G6">
-        <v>0.380110235072572</v>
+        <v>0.3895889495947642</v>
       </c>
       <c r="H6">
-        <v>0.2675740740740746</v>
+        <v>0.3099091880341884</v>
       </c>
       <c r="I6" s="2">
         <v>41518</v>
@@ -573,10 +573,10 @@
         <v>0.01715281745218458</v>
       </c>
       <c r="G7">
-        <v>-0.4042504123162414</v>
+        <v>-0.3756888419421722</v>
       </c>
       <c r="H7">
-        <v>-0.05668871252204566</v>
+        <v>-0.05548916207249555</v>
       </c>
       <c r="I7" s="2">
         <v>41760</v>
@@ -602,10 +602,10 @@
         <v>0.01271577675424276</v>
       </c>
       <c r="G8">
-        <v>0.3593949050992329</v>
+        <v>0.3380558456525704</v>
       </c>
       <c r="H8">
-        <v>-0.305615951178452</v>
+        <v>-0.2691754187170843</v>
       </c>
       <c r="I8" s="2">
         <v>41791</v>
@@ -631,10 +631,10 @@
         <v>0.01791180554656802</v>
       </c>
       <c r="G9">
-        <v>-0.2906000434898321</v>
+        <v>-0.2193203707738114</v>
       </c>
       <c r="H9">
-        <v>0.3245639329805994</v>
+        <v>0.3309881291547963</v>
       </c>
       <c r="I9" s="2">
         <v>41821</v>
@@ -660,10 +660,10 @@
         <v>0.0249056353204874</v>
       </c>
       <c r="G10">
-        <v>0.135526589879664</v>
+        <v>0.1089181737386391</v>
       </c>
       <c r="H10">
-        <v>0.1942895723104057</v>
+        <v>0.1654742186825509</v>
       </c>
       <c r="I10" s="2">
         <v>41852</v>
@@ -689,10 +689,10 @@
         <v>0.008712513813338929</v>
       </c>
       <c r="G11">
-        <v>0.2110892761291312</v>
+        <v>0.2205679906513234</v>
       </c>
       <c r="H11">
-        <v>0.07535185185185211</v>
+        <v>0.1176869658119659</v>
       </c>
       <c r="I11" s="2">
         <v>41883</v>
@@ -718,10 +718,10 @@
         <v>0.02259624092374374</v>
       </c>
       <c r="G12">
-        <v>-0.605190963546004</v>
+        <v>-0.5766293931719348</v>
       </c>
       <c r="H12">
-        <v>-0.1703791887125221</v>
+        <v>-0.169179638262972</v>
       </c>
       <c r="I12" s="2">
         <v>42125</v>
@@ -747,10 +747,10 @@
         <v>0.008959985126796383</v>
       </c>
       <c r="G13">
-        <v>0.2919777208342222</v>
+        <v>0.2706386613875598</v>
       </c>
       <c r="H13">
-        <v>0.007670762108261453</v>
+        <v>0.04411129456962914</v>
       </c>
       <c r="I13" s="2">
         <v>42156</v>
@@ -776,10 +776,10 @@
         <v>0.004902263324004508</v>
       </c>
       <c r="G14">
-        <v>-0.2443751607395184</v>
+        <v>-0.1730954880234976</v>
       </c>
       <c r="H14">
-        <v>-0.0109360670194012</v>
+        <v>-0.004511870845204324</v>
       </c>
       <c r="I14" s="2">
         <v>42186</v>
@@ -805,10 +805,10 @@
         <v>0.01118931736475592</v>
       </c>
       <c r="G15">
-        <v>0.5564421841312639</v>
+        <v>0.529833767990239</v>
       </c>
       <c r="H15">
-        <v>0.3334562389770728</v>
+        <v>0.304640885349218</v>
       </c>
       <c r="I15" s="2">
         <v>42217</v>
@@ -834,10 +834,10 @@
         <v>0.009935158164963043</v>
       </c>
       <c r="G16">
-        <v>0.07320347365999491</v>
+        <v>0.08268218818218709</v>
       </c>
       <c r="H16">
-        <v>0.2393269476372928</v>
+        <v>0.2816620615974066</v>
       </c>
       <c r="I16" s="2">
         <v>42248</v>
@@ -863,10 +863,10 @@
         <v>0.01392672628990896</v>
       </c>
       <c r="G17">
-        <v>0.05297616910388792</v>
+        <v>0.08153773947795706</v>
       </c>
       <c r="H17">
-        <v>0.264390926230007</v>
+        <v>0.2655904766795572</v>
       </c>
       <c r="I17" s="2">
         <v>42491</v>
@@ -892,10 +892,10 @@
         <v>0.02041042474488683</v>
       </c>
       <c r="G18">
-        <v>0.4138031176596195</v>
+        <v>0.392464058212957</v>
       </c>
       <c r="H18">
-        <v>-0.02643622286079239</v>
+        <v>0.0100043096005753</v>
       </c>
       <c r="I18" s="2">
         <v>42522</v>
@@ -921,10 +921,10 @@
         <v>0.007416364875281273</v>
       </c>
       <c r="G19">
-        <v>-0.08090440114048958</v>
+        <v>-0.00962472842446882</v>
       </c>
       <c r="H19">
-        <v>-0.1365471781305119</v>
+        <v>-0.130122981956315</v>
       </c>
       <c r="I19" s="2">
         <v>42552</v>
@@ -950,10 +950,10 @@
         <v>-0.0029944062002287</v>
       </c>
       <c r="G20">
-        <v>0.3934083632786776</v>
+        <v>0.3667999471376526</v>
       </c>
       <c r="H20">
-        <v>0.01487386349814557</v>
+        <v>-0.01394149012970924</v>
       </c>
       <c r="I20" s="2">
         <v>42583</v>
@@ -979,10 +979,10 @@
         <v>-0.01011195938975235</v>
       </c>
       <c r="G21">
-        <v>0.3975330169338391</v>
+        <v>0.4070117314560313</v>
       </c>
       <c r="H21">
-        <v>0.1795185185185186</v>
+        <v>0.2218536324786324</v>
       </c>
       <c r="I21" s="2">
         <v>42614</v>
@@ -1008,10 +1008,10 @@
         <v>0.003873199844137309</v>
       </c>
       <c r="G22">
-        <v>0.3910203201251372</v>
+        <v>0.4195818904992064</v>
       </c>
       <c r="H22">
-        <v>0.1785097001763671</v>
+        <v>0.1797092506259172</v>
       </c>
       <c r="I22" s="2">
         <v>42856</v>
@@ -1037,10 +1037,10 @@
         <v>0.008981392861905912</v>
       </c>
       <c r="G23">
-        <v>0.1136064608257934</v>
+        <v>0.09226740137913092</v>
       </c>
       <c r="H23">
-        <v>-0.1755023148148158</v>
+        <v>-0.1390617823534481</v>
       </c>
       <c r="I23" s="2">
         <v>42887</v>
@@ -1066,10 +1066,10 @@
         <v>0.01507386017091225</v>
       </c>
       <c r="G24">
-        <v>-0.314054558483968</v>
+        <v>-0.2427748857679473</v>
       </c>
       <c r="H24">
-        <v>-0.1758148548981886</v>
+        <v>-0.1693906587239917</v>
       </c>
       <c r="I24" s="2">
         <v>42917</v>
@@ -1095,10 +1095,10 @@
         <v>0.02380296459753059</v>
       </c>
       <c r="G25">
-        <v>0.2092266446142002</v>
+        <v>0.1826182284731752</v>
       </c>
       <c r="H25">
-        <v>0.1541903659611998</v>
+        <v>0.125375012333345</v>
       </c>
       <c r="I25" s="2">
         <v>42948</v>
@@ -1124,10 +1124,10 @@
         <v>0.01388945244713988</v>
       </c>
       <c r="G26">
-        <v>-0.1251616883770406</v>
+        <v>-0.1156829738548484</v>
       </c>
       <c r="H26">
-        <v>-0.3143703703703702</v>
+        <v>-0.2720352564102564</v>
       </c>
       <c r="I26" s="2">
         <v>42979</v>

</xml_diff>